<commit_message>
CI Reports [2026-06-25 19:49]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Feature Reports/CreateTicket.xlsx
+++ b/Test Execution Report/Feature Reports/CreateTicket.xlsx
@@ -2602,10 +2602,10 @@
         <v>Test should pass per acceptance criteria</v>
       </c>
       <c r="J45" t="str">
-        <v>_x001b_[31mTest timeout of 30000ms exceeded._x001b_[39m</v>
+        <v>Test passed successfully</v>
       </c>
       <c r="K45" t="str">
-        <v>NOT RUN</v>
+        <v>PASS</v>
       </c>
       <c r="L45" t="str">
         <v>Automation (Playwright)</v>

</xml_diff>